<commit_message>
v0.6.2: ruido con el Kc del trim, sin entrada xFz y panel de información visible
- El ruido IEC 60534-8-4 de líquidos toma el Kc del trim como inicio de cavitación (el mismo
  criterio que la alerta); el xFz típico solo se usa si Kc está en blanco.
- Se quita la entrada opcional xFz; xFzp1 queda como resultado informativo.
- La ventana ya no exige 1580 px de ancho: la columna izquierda se desplaza en horizontal y
  el panel de información queda entero a la vista en pantallas de 1280–1366 px.
- Planilla del kit y manual de trim regenerados.

Co-Authored-By: Claude Opus 5.5 (1M context) <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01U4yJ7uLSXttFganqs6AWmH
</commit_message>
<xml_diff>
--- a/kit_validacion/Planilla_comparacion_N25-Valves-Sizing.xlsx
+++ b/kit_validacion/Planilla_comparacion_N25-Valves-Sizing.xlsx
@@ -873,7 +873,7 @@
         </is>
       </c>
       <c r="E7" s="4" t="n">
-        <v>93.3</v>
+        <v>80.3</v>
       </c>
       <c r="F7" s="5" t="n"/>
       <c r="G7" s="5" t="n"/>
@@ -4313,7 +4313,7 @@
         </is>
       </c>
       <c r="E97" s="4" t="n">
-        <v>80.7</v>
+        <v>77.59999999999999</v>
       </c>
       <c r="F97" s="5" t="n"/>
       <c r="G97" s="5" t="n"/>
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="E98" s="4" t="n">
-        <v>84</v>
+        <v>79.40000000000001</v>
       </c>
       <c r="F98" s="5" t="n"/>
       <c r="G98" s="5" t="n"/>
@@ -4393,7 +4393,7 @@
         </is>
       </c>
       <c r="E99" s="4" t="n">
-        <v>84</v>
+        <v>76.59999999999999</v>
       </c>
       <c r="F99" s="5" t="n"/>
       <c r="G99" s="5" t="n"/>

</xml_diff>